<commit_message>
Added new upscale R file, where multiple images processed at once
</commit_message>
<xml_diff>
--- a/image14_Cluster_Plastics_GFP_CenterIntensity.xlsx
+++ b/image14_Cluster_Plastics_GFP_CenterIntensity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrewchang/Desktop/Medical School!/Research/R For Data Science/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrewchang/Desktop/Medical School/Research/R For Data Science/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1806C8BB-A5BB-A847-B184-5A00412246FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CABB581-75F9-1F4B-B1E9-DB95EF052E86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="760" windowWidth="27800" windowHeight="15620" xr2:uid="{AFBA743E-F5DB-244D-9B58-7FE4040EE853}"/>
+    <workbookView xWindow="6720" yWindow="7860" windowWidth="27800" windowHeight="15620" xr2:uid="{AFBA743E-F5DB-244D-9B58-7FE4040EE853}"/>
   </bookViews>
   <sheets>
     <sheet name="Selection" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="13">
   <si>
     <t/>
   </si>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t>cluster plastics</t>
+  </si>
+  <si>
+    <t>Selection</t>
   </si>
 </sst>
 </file>
@@ -131,7 +134,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -140,6 +143,9 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -481,7 +487,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52FBB9F3-EBED-B94E-8F0A-5010ED7EDFFE}">
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" outlineLevelRow="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="11" style="3" customWidth="1"/>
@@ -489,62 +495,41 @@
     <col min="9" max="256" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A1" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="2" customFormat="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.15">
-      <c r="A2" s="3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A3" s="3">
         <v>1520</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="1">
-        <v>2</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="1">
-        <v>1</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="3">
-        <v>1549</v>
-      </c>
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -564,12 +549,12 @@
         <v>11</v>
       </c>
       <c r="H3" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A4" s="3">
-        <v>177</v>
+        <v>1549</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>0</v>
@@ -590,12 +575,12 @@
         <v>11</v>
       </c>
       <c r="H4" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A5" s="3">
-        <v>354</v>
+        <v>177</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>0</v>
@@ -616,12 +601,12 @@
         <v>11</v>
       </c>
       <c r="H5" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A6" s="3">
-        <v>273</v>
+        <v>354</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>0</v>
@@ -642,12 +627,12 @@
         <v>11</v>
       </c>
       <c r="H6" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A7" s="3">
-        <v>482</v>
+        <v>273</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>0</v>
@@ -668,12 +653,12 @@
         <v>11</v>
       </c>
       <c r="H7" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A8" s="3">
-        <v>350</v>
+        <v>482</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>0</v>
@@ -694,12 +679,12 @@
         <v>11</v>
       </c>
       <c r="H8" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A9" s="3">
-        <v>194</v>
+        <v>350</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>0</v>
@@ -720,12 +705,12 @@
         <v>11</v>
       </c>
       <c r="H9" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A10" s="3">
-        <v>142</v>
+        <v>194</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>0</v>
@@ -746,12 +731,12 @@
         <v>11</v>
       </c>
       <c r="H10" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A11" s="3">
-        <v>313</v>
+        <v>142</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>0</v>
@@ -772,12 +757,12 @@
         <v>11</v>
       </c>
       <c r="H11" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3">
-        <v>222</v>
+        <v>313</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>0</v>
@@ -798,12 +783,12 @@
         <v>11</v>
       </c>
       <c r="H12" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>0</v>
@@ -824,12 +809,12 @@
         <v>11</v>
       </c>
       <c r="H13" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3">
-        <v>234</v>
+        <v>217</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>0</v>
@@ -850,12 +835,12 @@
         <v>11</v>
       </c>
       <c r="H14" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A15" s="3">
-        <v>145</v>
+        <v>234</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>0</v>
@@ -876,12 +861,12 @@
         <v>11</v>
       </c>
       <c r="H15" s="1">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A16" s="3">
-        <v>197</v>
+        <v>145</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>0</v>
@@ -902,12 +887,12 @@
         <v>11</v>
       </c>
       <c r="H16" s="1">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A17" s="3">
-        <v>233</v>
+        <v>197</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>0</v>
@@ -928,12 +913,12 @@
         <v>11</v>
       </c>
       <c r="H17" s="1">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A18" s="3">
-        <v>616</v>
+        <v>233</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>0</v>
@@ -954,12 +939,12 @@
         <v>11</v>
       </c>
       <c r="H18" s="1">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A19" s="3">
-        <v>397</v>
+        <v>616</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>0</v>
@@ -980,12 +965,12 @@
         <v>11</v>
       </c>
       <c r="H19" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A20" s="3">
-        <v>129</v>
+        <v>397</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>0</v>
@@ -1006,12 +991,12 @@
         <v>11</v>
       </c>
       <c r="H20" s="1">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A21" s="3">
-        <v>172</v>
+        <v>129</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>0</v>
@@ -1032,12 +1017,12 @@
         <v>11</v>
       </c>
       <c r="H21" s="1">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A22" s="3">
-        <v>202</v>
+        <v>172</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>0</v>
@@ -1058,12 +1043,12 @@
         <v>11</v>
       </c>
       <c r="H22" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A23" s="3">
-        <v>302</v>
+        <v>202</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>0</v>
@@ -1084,12 +1069,12 @@
         <v>11</v>
       </c>
       <c r="H23" s="1">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A24" s="3">
-        <v>193</v>
+        <v>302</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>0</v>
@@ -1110,12 +1095,12 @@
         <v>11</v>
       </c>
       <c r="H24" s="1">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A25" s="3">
-        <v>274</v>
+        <v>193</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>0</v>
@@ -1136,12 +1121,12 @@
         <v>11</v>
       </c>
       <c r="H25" s="1">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="26" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A26" s="3">
-        <v>490</v>
+        <v>274</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>0</v>
@@ -1162,12 +1147,12 @@
         <v>11</v>
       </c>
       <c r="H26" s="1">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="27" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A27" s="3">
-        <v>148</v>
+        <v>490</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>0</v>
@@ -1188,12 +1173,12 @@
         <v>11</v>
       </c>
       <c r="H27" s="1">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="28" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A28" s="3">
-        <v>281</v>
+        <v>148</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>0</v>
@@ -1214,12 +1199,12 @@
         <v>11</v>
       </c>
       <c r="H28" s="1">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A29" s="3">
-        <v>620</v>
+        <v>281</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>0</v>
@@ -1240,12 +1225,12 @@
         <v>11</v>
       </c>
       <c r="H29" s="1">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="30" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A30" s="3">
-        <v>151</v>
+        <v>620</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>0</v>
@@ -1266,12 +1251,12 @@
         <v>11</v>
       </c>
       <c r="H30" s="1">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A31" s="3">
-        <v>173</v>
+        <v>151</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>0</v>
@@ -1292,12 +1277,12 @@
         <v>11</v>
       </c>
       <c r="H31" s="1">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="32" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A32" s="3">
-        <v>478</v>
+        <v>173</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>0</v>
@@ -1318,12 +1303,12 @@
         <v>11</v>
       </c>
       <c r="H32" s="1">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="33" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A33" s="3">
-        <v>688</v>
+        <v>478</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>0</v>
@@ -1344,12 +1329,12 @@
         <v>11</v>
       </c>
       <c r="H33" s="1">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A34" s="3">
-        <v>772</v>
+        <v>688</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>0</v>
@@ -1370,12 +1355,12 @@
         <v>11</v>
       </c>
       <c r="H34" s="1">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A35" s="3">
-        <v>1286</v>
+        <v>772</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>0</v>
@@ -1396,12 +1381,12 @@
         <v>11</v>
       </c>
       <c r="H35" s="1">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="36" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A36" s="3">
-        <v>188</v>
+        <v>1286</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>0</v>
@@ -1422,12 +1407,12 @@
         <v>11</v>
       </c>
       <c r="H36" s="1">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="37" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A37" s="3">
-        <v>908</v>
+        <v>188</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>0</v>
@@ -1448,12 +1433,12 @@
         <v>11</v>
       </c>
       <c r="H37" s="1">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="38" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A38" s="3">
-        <v>277</v>
+        <v>908</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>0</v>
@@ -1474,12 +1459,12 @@
         <v>11</v>
       </c>
       <c r="H38" s="1">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="39" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A39" s="3">
-        <v>159</v>
+        <v>277</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>0</v>
@@ -1500,12 +1485,12 @@
         <v>11</v>
       </c>
       <c r="H39" s="1">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="40" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A40" s="3">
-        <v>230</v>
+        <v>159</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>0</v>
@@ -1526,12 +1511,12 @@
         <v>11</v>
       </c>
       <c r="H40" s="1">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="41" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A41" s="3">
-        <v>1130</v>
+        <v>230</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>0</v>
@@ -1552,12 +1537,12 @@
         <v>11</v>
       </c>
       <c r="H41" s="1">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="42" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A42" s="3">
-        <v>647</v>
+        <v>1130</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>0</v>
@@ -1578,12 +1563,12 @@
         <v>11</v>
       </c>
       <c r="H42" s="1">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="43" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A43" s="3">
-        <v>665</v>
+        <v>647</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>0</v>
@@ -1604,12 +1589,12 @@
         <v>11</v>
       </c>
       <c r="H43" s="1">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A44" s="3">
-        <v>547</v>
+        <v>665</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>0</v>
@@ -1630,12 +1615,12 @@
         <v>11</v>
       </c>
       <c r="H44" s="1">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="45" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A45" s="3">
-        <v>542</v>
+        <v>547</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>0</v>
@@ -1656,12 +1641,12 @@
         <v>11</v>
       </c>
       <c r="H45" s="1">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="46" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A46" s="3">
-        <v>377</v>
+        <v>542</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>0</v>
@@ -1682,12 +1667,12 @@
         <v>11</v>
       </c>
       <c r="H46" s="1">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="47" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A47" s="3">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>0</v>
@@ -1708,12 +1693,12 @@
         <v>11</v>
       </c>
       <c r="H47" s="1">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="48" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A48" s="3">
-        <v>152</v>
+        <v>375</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>0</v>
@@ -1734,32 +1719,58 @@
         <v>11</v>
       </c>
       <c r="H48" s="1">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="49" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
       <c r="A49" s="3">
+        <v>152</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D49" s="1">
+        <v>2</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F49" s="1">
+        <v>1</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H49" s="1">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" collapsed="1" x14ac:dyDescent="0.15">
+      <c r="A50" s="3">
         <v>446</v>
       </c>
-      <c r="B49" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D49" s="1">
-        <v>2</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F49" s="1">
-        <v>1</v>
-      </c>
-      <c r="G49" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H49" s="1">
+      <c r="B50" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D50" s="1">
+        <v>2</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F50" s="1">
+        <v>1</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H50" s="1">
         <v>47</v>
       </c>
     </row>

</xml_diff>